<commit_message>
study.xlsx: drop DM's categorical row, which only restated the default
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/extdata/ard-spec/study.xlsx
+++ b/inst/extdata/ard-spec/study.xlsx
@@ -1515,7 +1515,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -1678,17 +1678,22 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>DM</t>
+          <t>ORR</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>categorical</t>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>{n:.0f} ({p:.1f%})</t>
+          <t>{N:.0f}</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1705,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>orr_ci</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1708,9 +1713,14 @@
           <t>1</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>n == 0</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>{N:.0f}</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -1732,12 +1742,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>n == 0</t>
+          <t>estimate == 1</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>{n:.0f} (100)</t>
         </is>
       </c>
     </row>
@@ -1757,14 +1767,9 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>estimate == 1</t>
-        </is>
-      </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>{n:.0f} (100)</t>
+          <t>{n:.0f} ({estimate:.1f%})</t>
         </is>
       </c>
     </row>
@@ -1781,32 +1786,10 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
-        <is>
-          <t>{n:.0f} ({estimate:.1f%})</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>ORR</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>orr_ci</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
         <is>
           <t>{conf.low:.1f%}, {conf.high:.1f%}</t>
         </is>

</xml_diff>